<commit_message>
feat: sync manually downloaded paper 71 (sciimmunol.adf9988)
</commit_message>
<xml_diff>
--- a/db/cellxgene/cellxgene_filtered/pns_papers_summary.xlsx
+++ b/db/cellxgene/cellxgene_filtered/pns_papers_summary.xlsx
@@ -4505,7 +4505,12 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>D:\OneDrive\Desktop\组\db\cellxgene\cellxgene_filtered\downloads\PMID_38100545_Early human lung immune cell development and its role in epithelial cell fate..pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: sync manually downloaded paper 12, 14, 55 (from recent folder check)
</commit_message>
<xml_diff>
--- a/db/cellxgene/cellxgene_filtered/pns_papers_summary.xlsx
+++ b/db/cellxgene/cellxgene_filtered/pns_papers_summary.xlsx
@@ -1472,7 +1472,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>D:\OneDrive\Desktop\组\db\cellxgene\cellxgene_filtered\downloads\PMID_36796082_A Unique Cellular Organization of Human Distal Airways and Its Disarray in Chronic Obstructive Pulmonary Disease..pdf</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1576,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Error</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -3688,7 +3693,12 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>D:\OneDrive\Desktop\组\db\cellxgene\cellxgene_filtered\downloads\PMID_39789339_Author Correction_ Progressive plasticity during colorectal cancer metastasis..pdf</t>
         </is>
       </c>
     </row>

</xml_diff>